<commit_message>
Adding CSV and dataframe libraries
</commit_message>
<xml_diff>
--- a/data/FlucIE_ProcessedData.xlsx
+++ b/data/FlucIE_ProcessedData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20411"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juliechen/Documents/UROP/TASEP/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ChemeGrad2021\Documents\Braatz Group\MRNA Synthesis\TASEP\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9FEF95FF-2EA9-6D4C-BE26-EF54CD83506D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D683D00-1E83-4868-947C-F4B86154A8F1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1300" windowWidth="27640" windowHeight="16940" xr2:uid="{6B94D0B7-30F9-8446-A036-BFF6193C6223}"/>
+    <workbookView xWindow="1500" yWindow="1296" windowWidth="27636" windowHeight="16944" xr2:uid="{6B94D0B7-30F9-8446-A036-BFF6193C6223}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,17 +20,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -78,7 +67,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -448,13 +437,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84FA570C-ABF3-3D41-82F4-FDB4E6F5488E}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -465,7 +454,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -479,7 +468,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -493,7 +482,7 @@
         <v>8.8000000000000007</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -507,7 +496,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -521,7 +510,7 @@
         <v>16.100000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -535,7 +524,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -549,7 +538,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -563,7 +552,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -577,7 +566,7 @@
         <v>9.1999999999999993</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>10</v>
       </c>

</xml_diff>